<commit_message>
feat(billing): implementar plan FREE con paywall a 25 facturas, sincronizacion directa Stripe API y exportadores ERP alineados
</commit_message>
<xml_diff>
--- a/output_pilot/CONTASOL_CLIENTE3.xlsx
+++ b/output_pilot/CONTASOL_CLIENTE3.xlsx
@@ -524,7 +524,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>430ST-091</t>
+          <t>4300ST091</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>430ST-091</t>
+          <t>4300ST091</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>430ST-088</t>
+          <t>4300ST088</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>430ST-088</t>
+          <t>4300ST088</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">

</xml_diff>